<commit_message>
fix: align e2e reference on transposition root cause
</commit_message>
<xml_diff>
--- a/tests/e2e/output/engagement/output/ar_gl_reconciliation.xlsx
+++ b/tests/e2e/output/engagement/output/ar_gl_reconciliation.xlsx
@@ -535,7 +535,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>inv-19877 (Stonebridge Market) treated as a probable digit-transposition (45,000 recorded vs 54,000 true) based on exact-amount + direction fit against the residual; NOT independently confirmed by a third source (no Stonebridge contract/invoice in data room) -- see open items.</t>
+          <t>inv-19877 (Stonebridge Market) treated as a probable digit-transposition in the GL control balance: the subledger records 45,000 and is believed correct; the GL is consistent with this invoice contributing 54,000 instead -- based on exact-amount + direction fit against the residual, NOT independently confirmed by a third source (no Stonebridge contract/invoice in data room) -- see open items.</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -761,7 +761,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Add: probable transposition correction - inv-19877 Stonebridge Market recorded as 45,000.00; digit-swap to 54,000.00 exactly closes residual in the required direction</t>
+          <t>Add: probable transposition correction - inv-19877 Stonebridge Market recorded (and believed correct) as 45,000.00 in the subledger; GL keyed the invoice as 54,000.00, a probable digit-swap error in the GL that exactly closes the residual in the required direction</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
@@ -769,7 +769,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GL higher than subledger (subledger understated)</t>
+          <t>GL higher than subledger (GL overstated / subledger believed correct)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>